<commit_message>
atualização botão Matriz Experimental
</commit_message>
<xml_diff>
--- a/replicas_template.xlsx
+++ b/replicas_template.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="27">
   <si>
     <t xml:space="preserve">Exp</t>
   </si>
@@ -46,25 +46,61 @@
     <t xml:space="preserve">86.0</t>
   </si>
   <si>
+    <t xml:space="preserve">85.5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">85.1</t>
+  </si>
+  <si>
     <t xml:space="preserve">68.9</t>
   </si>
   <si>
+    <t xml:space="preserve">68.4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">68.7</t>
+  </si>
+  <si>
     <t xml:space="preserve">81.0</t>
   </si>
   <si>
+    <t xml:space="preserve">81.1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">79.9</t>
+  </si>
+  <si>
     <t xml:space="preserve">73.6</t>
   </si>
   <si>
+    <t xml:space="preserve">73.2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">73.4</t>
+  </si>
+  <si>
     <t xml:space="preserve">78.6</t>
   </si>
   <si>
+    <t xml:space="preserve">78.2</t>
+  </si>
+  <si>
     <t xml:space="preserve">53.3</t>
   </si>
   <si>
     <t xml:space="preserve">82.0</t>
   </si>
   <si>
+    <t xml:space="preserve">82.3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">82.7</t>
+  </si>
+  <si>
     <t xml:space="preserve">63.6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">63.5</t>
   </si>
 </sst>
 </file>
@@ -154,13 +190,17 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
       <alignment horizontal="center" vertical="top" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
   </cellXfs>
@@ -373,129 +413,129 @@
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="0" t="n">
+      <c r="A2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="0" t="s">
+      <c r="B2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C2" s="0" t="s">
+      <c r="C2" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="0" t="s">
+      <c r="D2" s="2" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="0" t="n">
+      <c r="A3" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="0" t="s">
+      <c r="B3" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="0" t="s">
+      <c r="C3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>78</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="D3" s="0" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="0" t="n">
-        <v>3</v>
-      </c>
-      <c r="B4" s="0" t="s">
+      <c r="B8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="C4" s="0" t="s">
-        <v>8</v>
-      </c>
-      <c r="D4" s="0" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="0" t="n">
-        <v>4</v>
-      </c>
-      <c r="B5" s="0" t="s">
+      <c r="B9" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="2" t="n">
         <v>9</v>
       </c>
-      <c r="C5" s="0" t="s">
-        <v>9</v>
-      </c>
-      <c r="D5" s="0" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="0" t="n">
-        <v>5</v>
-      </c>
-      <c r="B6" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="C6" s="0" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" s="0" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="0" t="n">
-        <v>6</v>
-      </c>
-      <c r="B7" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="C7" s="0" t="s">
-        <v>11</v>
-      </c>
-      <c r="D7" s="0" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="0" t="n">
-        <v>7</v>
-      </c>
-      <c r="B8" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="C8" s="0" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="0" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="0" t="n">
-        <v>8</v>
-      </c>
-      <c r="B9" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="C9" s="0" t="s">
-        <v>13</v>
-      </c>
-      <c r="D9" s="0" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="0" t="n">
-        <v>9</v>
-      </c>
-      <c r="B10" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="C10" s="0" t="s">
-        <v>14</v>
-      </c>
-      <c r="D10" s="0" t="s">
-        <v>14</v>
+      <c r="B10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>26</v>
       </c>
     </row>
   </sheetData>

</xml_diff>